<commit_message>
refactor: update document title and reformat HTML structure for consistency
</commit_message>
<xml_diff>
--- a/批量下单脚本/订单分表模版.xlsx
+++ b/批量下单脚本/订单分表模版.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9420" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="9420"/>
   </bookViews>
   <sheets>
     <sheet name="订单" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="56">
   <si>
     <t>导入编号</t>
   </si>
@@ -100,6 +100,9 @@
     <t>客服备注</t>
   </si>
   <si>
+    <t>客户备注</t>
+  </si>
+  <si>
     <t>客户账号</t>
   </si>
   <si>
@@ -170,168 +173,6 @@
   </si>
   <si>
     <t>单价</t>
-  </si>
-  <si>
-    <t>纸张宽度</t>
-  </si>
-  <si>
-    <t>GP-C180I（USB+网口+钱箱）</t>
-  </si>
-  <si>
-    <t>6970362037798</t>
-  </si>
-  <si>
-    <t>TX-180</t>
-  </si>
-  <si>
-    <t>黑色USB+网口+钱箱接口</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>98</t>
-  </si>
-  <si>
-    <t>GP-C180I（USB+网口）</t>
-  </si>
-  <si>
-    <t>6970362037799</t>
-  </si>
-  <si>
-    <t>黑色USB+网口</t>
-  </si>
-  <si>
-    <t>95</t>
-  </si>
-  <si>
-    <t>XP-C260M（USB+网口）</t>
-  </si>
-  <si>
-    <t>6974657411974</t>
-  </si>
-  <si>
-    <t>XP-00012</t>
-  </si>
-  <si>
-    <t>245</t>
-  </si>
-  <si>
-    <t>XP-T80Q（USB+WIFI）</t>
-  </si>
-  <si>
-    <t>6974657413404</t>
-  </si>
-  <si>
-    <t>XP-8068</t>
-  </si>
-  <si>
-    <t>USB+WIFI（局域网）</t>
-  </si>
-  <si>
-    <t>XP-T503（USB+WIFI+蓝牙）</t>
-  </si>
-  <si>
-    <t>6974657412537</t>
-  </si>
-  <si>
-    <t>XP-12</t>
-  </si>
-  <si>
-    <t>USB+WIFI（云）+蓝牙</t>
-  </si>
-  <si>
-    <t>XP-T503（USB+4G+蓝牙）</t>
-  </si>
-  <si>
-    <t>6974657414623</t>
-  </si>
-  <si>
-    <t>USB+4G+蓝牙</t>
-  </si>
-  <si>
-    <t>XP-C503（USB+WIFI+蓝牙）</t>
-  </si>
-  <si>
-    <t>6974657413046</t>
-  </si>
-  <si>
-    <t>XP-124</t>
-  </si>
-  <si>
-    <t>XP-C503（USB+4G+蓝牙）</t>
-  </si>
-  <si>
-    <t>6974657413053</t>
-  </si>
-  <si>
-    <t>XP-T271U（USB+WIFI+蓝牙）</t>
-  </si>
-  <si>
-    <t>6974657413138</t>
-  </si>
-  <si>
-    <t>BT033</t>
-  </si>
-  <si>
-    <t>黑白USB+WIFI（云）+蓝牙</t>
-  </si>
-  <si>
-    <t>XP-T271U（USB+4G+蓝牙）</t>
-  </si>
-  <si>
-    <t>6974657410137</t>
-  </si>
-  <si>
-    <t>黑白USB+蓝牙+4G（云）</t>
-  </si>
-  <si>
-    <t>XP-58IINT（USB+WIFI）</t>
-  </si>
-  <si>
-    <t>6974657412629</t>
-  </si>
-  <si>
-    <t>XP-580045</t>
-  </si>
-  <si>
-    <t>黑黄USB+WIFI（云）</t>
-  </si>
-  <si>
-    <t>M80-CW（USB+WIFI）</t>
-  </si>
-  <si>
-    <t>M80CW001</t>
-  </si>
-  <si>
-    <t>XP-8054</t>
-  </si>
-  <si>
-    <t>USB+WIFI（云）</t>
-  </si>
-  <si>
-    <t>328</t>
-  </si>
-  <si>
-    <t>80*60纸</t>
-  </si>
-  <si>
-    <t>TXXPZ101</t>
-  </si>
-  <si>
-    <t>RM-0007</t>
-  </si>
-  <si>
-    <t>1.5</t>
-  </si>
-  <si>
-    <t>57*50纸</t>
-  </si>
-  <si>
-    <t>TXXPZ002</t>
-  </si>
-  <si>
-    <t>RM-0002</t>
   </si>
   <si>
     <t>（上海商米）D3PRO单屏</t>
@@ -505,7 +346,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -521,41 +362,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="4"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFFC000"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="9"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <name val="宋体"/>
       <charset val="134"/>
     </font>
@@ -588,6 +394,13 @@
       <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1076,10 +889,10 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1088,206 +901,179 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1609,167 +1395,173 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr defaultColWidth="10.6296296296296" defaultRowHeight="37" customHeight="1" outlineLevelRow="5"/>
   <cols>
-    <col min="1" max="1" width="22.25" style="16" customWidth="1"/>
-    <col min="2" max="2" width="8.25" style="16" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5" style="16" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="30.7777777777778" style="16" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="32.4444444444444" style="16" customWidth="1"/>
-    <col min="6" max="6" width="10.6296296296296" style="16" customWidth="1"/>
-    <col min="7" max="7" width="10.5" style="16" customWidth="1"/>
-    <col min="8" max="8" width="15" style="16" customWidth="1"/>
-    <col min="9" max="9" width="22" style="16" customWidth="1"/>
-    <col min="10" max="10" width="23.3333333333333" style="16" customWidth="1"/>
-    <col min="11" max="11" width="17.5555555555556" style="16" customWidth="1"/>
-    <col min="12" max="15" width="24.6666666666667" style="16" customWidth="1"/>
-    <col min="16" max="16" width="24.6666666666667" style="17" customWidth="1"/>
-    <col min="17" max="17" width="35.8796296296296" style="16" customWidth="1"/>
-    <col min="18" max="16384" width="10.6296296296296" style="16"/>
+    <col min="1" max="1" width="22.25" style="7" customWidth="1"/>
+    <col min="2" max="2" width="8.25" style="7" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5" style="7" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="30.7777777777778" style="7" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="32.4444444444444" style="7" customWidth="1"/>
+    <col min="6" max="6" width="10.6296296296296" style="7" customWidth="1"/>
+    <col min="7" max="7" width="10.5" style="7" customWidth="1"/>
+    <col min="8" max="9" width="15" style="7" customWidth="1"/>
+    <col min="10" max="10" width="22" style="7" customWidth="1"/>
+    <col min="11" max="11" width="23.3333333333333" style="7" customWidth="1"/>
+    <col min="12" max="12" width="17.5555555555556" style="7" customWidth="1"/>
+    <col min="13" max="16" width="24.6666666666667" style="7" customWidth="1"/>
+    <col min="17" max="17" width="24.6666666666667" style="8" customWidth="1"/>
+    <col min="18" max="18" width="35.8796296296296" style="7" customWidth="1"/>
+    <col min="19" max="16384" width="10.6296296296296" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" s="15" customFormat="1" customHeight="1" spans="1:16">
-      <c r="A1" s="18" t="s">
+    <row r="1" s="6" customFormat="1" customHeight="1" spans="1:17">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="J1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="K1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="18" t="s">
+      <c r="L1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="15" t="s">
+      <c r="M1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="N1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="15" t="s">
+      <c r="O1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="18" t="s">
+      <c r="P1" s="6" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="9" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" customHeight="1" spans="1:17">
-      <c r="A2" s="19"/>
-      <c r="E2" s="20"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" s="16" t="s">
+    <row r="2" customHeight="1" spans="1:18">
+      <c r="A2" s="10"/>
+      <c r="E2" s="11"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="K2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="16" t="s">
+      <c r="L2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="P2" s="23" t="s">
+      <c r="M2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="Q2" s="24"/>
+      <c r="Q2" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="R2" s="15"/>
     </row>
-    <row r="3" customHeight="1" spans="5:16">
-      <c r="E3" s="21"/>
-      <c r="I3" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" s="16" t="s">
+    <row r="3" customHeight="1" spans="5:17">
+      <c r="E3" s="12"/>
+      <c r="J3" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="L3" s="16" t="s">
+      <c r="L3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q3" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="P3" s="23" t="s">
-        <v>20</v>
-      </c>
     </row>
-    <row r="4" customHeight="1" spans="8:16">
-      <c r="H4" s="22"/>
-      <c r="I4" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4" s="16" t="s">
+    <row r="4" customHeight="1" spans="8:17">
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="L4" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="P4" s="23" t="s">
-        <v>20</v>
+      <c r="L4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="14" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="9:16">
-      <c r="I5" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" s="16" t="s">
+    <row r="5" customHeight="1" spans="10:17">
+      <c r="J5" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="16" t="s">
+      <c r="K5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="L5" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="P5" s="23" t="s">
-        <v>20</v>
+      <c r="L5" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q5" s="14" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="6" customHeight="1" spans="8:16">
-      <c r="H6" s="22"/>
-      <c r="I6" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6" s="16" t="s">
+    <row r="6" customHeight="1" spans="8:17">
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="16" t="s">
+      <c r="K6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="L6" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="P6" s="23" t="s">
-        <v>20</v>
+      <c r="L6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q6" s="14" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1783,484 +1575,158 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelCol="7"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelRow="6" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="20.6296296296296" style="2" customWidth="1"/>
-    <col min="2" max="2" width="29.3333333333333" style="2" customWidth="1"/>
-    <col min="3" max="3" width="14.5" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.2222222222222" style="1" customWidth="1"/>
-    <col min="5" max="5" width="26.3796296296296" style="1" customWidth="1"/>
-    <col min="6" max="7" width="10.6296296296296" style="1"/>
-    <col min="8" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="20.6296296296296" style="1" customWidth="1"/>
+    <col min="2" max="2" width="29.3333333333333" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.2222222222222" style="2" customWidth="1"/>
+    <col min="5" max="5" width="26.3796296296296" style="2" customWidth="1"/>
+    <col min="6" max="7" width="10.6296296296296" style="2"/>
+    <col min="8" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.6" spans="1:8">
+    <row r="1" ht="15.6" spans="1:7">
       <c r="A1" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H1" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5" t="s">
+    <row r="2" spans="2:7">
+      <c r="B2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5">
+        <v>1680</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7">
+      <c r="B3" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="C3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H2" s="1">
+      <c r="D3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1</v>
+      </c>
+      <c r="G3" s="5">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7">
+      <c r="B4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1</v>
+      </c>
+      <c r="G4" s="5">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7">
+      <c r="B5" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7">
+      <c r="B6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1</v>
+      </c>
+      <c r="G6" s="5">
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="H3" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" spans="2:8">
-      <c r="B4" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="2:8">
-      <c r="B5" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" s="10">
+    <row r="7" spans="2:7">
+      <c r="B7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="2">
         <v>1</v>
       </c>
-      <c r="G5" s="10">
-        <v>195</v>
-      </c>
-      <c r="H5" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8">
-      <c r="B6" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="5">
-        <v>1</v>
-      </c>
-      <c r="G6" s="5">
-        <v>255</v>
-      </c>
-      <c r="H6" s="1">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8">
-      <c r="B7" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="F7" s="5">
-        <v>1</v>
-      </c>
       <c r="G7" s="5">
-        <v>245</v>
-      </c>
-      <c r="H7" s="1">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8">
-      <c r="B8" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" s="5">
-        <v>1</v>
-      </c>
-      <c r="G8" s="5">
-        <v>295</v>
-      </c>
-      <c r="H8" s="1">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8">
-      <c r="B9" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="F9" s="5">
-        <v>1</v>
-      </c>
-      <c r="G9" s="5">
-        <v>285</v>
-      </c>
-      <c r="H9" s="1">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7">
-      <c r="B10" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="F10" s="5">
-        <v>1</v>
-      </c>
-      <c r="G10" s="5">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7">
-      <c r="B11" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="F11" s="5">
-        <v>1</v>
-      </c>
-      <c r="G11" s="5">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8">
-      <c r="B12" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="F12" s="5">
-        <v>1</v>
-      </c>
-      <c r="G12" s="5">
-        <v>150</v>
-      </c>
-      <c r="H12" s="1">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8">
-      <c r="B13" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="H13" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="14" s="1" customFormat="1" spans="1:8">
-      <c r="A14" s="4"/>
-      <c r="B14" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="H14" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" s="1" customFormat="1" spans="1:8">
-      <c r="A15" s="4"/>
-      <c r="B15" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F15" s="1">
-        <v>1</v>
-      </c>
-      <c r="G15" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="H15" s="1">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7">
-      <c r="B16" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="F16" s="1">
-        <v>1</v>
-      </c>
-      <c r="G16" s="14">
-        <v>1680</v>
-      </c>
-    </row>
-    <row r="17" spans="2:8">
-      <c r="B17" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="F17" s="1">
-        <v>1</v>
-      </c>
-      <c r="G17" s="14">
-        <v>280</v>
-      </c>
-      <c r="H17" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7">
-      <c r="B18" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="F18" s="1">
-        <v>1</v>
-      </c>
-      <c r="G18" s="14">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7">
-      <c r="B19" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="F19" s="1">
-        <v>1</v>
-      </c>
-      <c r="G19" s="14">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7">
-      <c r="B20" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="F20" s="1">
-        <v>1</v>
-      </c>
-      <c r="G20" s="14">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7">
-      <c r="B21" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="F21" s="1">
-        <v>1</v>
-      </c>
-      <c r="G21" s="14">
         <v>1050</v>
       </c>
     </row>

</xml_diff>